<commit_message>
egzamin.xlsx: zestawienie do sprawozdania – data wydanego zaświadczenia w kolumnie F
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/documents/templates/egzamin.xlsx
+++ b/backend/documents/templates/egzamin.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr codeName="Ten_skoroszyt" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/patrykkarpinski/Wszystko/Projekty Programowanie/McMed/backend/documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D82C472-AD97-5E40-A2A2-A8D2808A8A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EF2503-E957-9A4C-857C-321F0277AEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" tabRatio="890" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16940" tabRatio="890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EGZ Teoria" sheetId="1" r:id="rId1"/>
@@ -418,7 +418,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -457,17 +457,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -575,17 +564,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -681,16 +659,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -700,29 +678,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -734,21 +709,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -756,49 +716,49 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -812,16 +772,13 @@
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -841,42 +798,32 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -891,6 +838,48 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1227,38 +1216,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A2" s="66"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A3" s="66"/>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
@@ -1268,7 +1257,7 @@
       <c r="B4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="63">
+      <c r="C4" s="54">
         <v>46204</v>
       </c>
       <c r="E4" t="s">
@@ -1279,11 +1268,11 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="68"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="74"/>
       <c r="D6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1295,257 +1284,257 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="19" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="64" t="s">
+      <c r="E7" s="55" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="62"/>
+      <c r="H7" s="53"/>
     </row>
     <row r="8" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="19"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
       <c r="D8" s="9"/>
-      <c r="E8" s="64"/>
+      <c r="E8" s="55"/>
       <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="19"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
       <c r="D9" s="9"/>
-      <c r="E9" s="64"/>
+      <c r="E9" s="55"/>
       <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="19"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
       <c r="D10" s="9"/>
-      <c r="E10" s="64"/>
+      <c r="E10" s="55"/>
       <c r="F10" s="9"/>
-      <c r="I10" s="62"/>
+      <c r="I10" s="53"/>
     </row>
     <row r="11" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="19"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
       <c r="D11" s="9"/>
-      <c r="E11" s="64"/>
+      <c r="E11" s="55"/>
       <c r="F11" s="9"/>
     </row>
     <row r="12" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="19"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
       <c r="D12" s="9"/>
-      <c r="E12" s="64"/>
+      <c r="E12" s="55"/>
       <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="19"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="64"/>
+      <c r="E13" s="55"/>
       <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
       <c r="D14" s="9"/>
-      <c r="E14" s="64"/>
+      <c r="E14" s="55"/>
       <c r="F14" s="9"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="19"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
       <c r="D15" s="9"/>
-      <c r="E15" s="64"/>
+      <c r="E15" s="55"/>
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="19"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
       <c r="D16" s="11"/>
-      <c r="E16" s="64"/>
+      <c r="E16" s="55"/>
       <c r="F16" s="11"/>
     </row>
     <row r="17" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="19"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
       <c r="D17" s="7"/>
-      <c r="E17" s="64"/>
+      <c r="E17" s="55"/>
       <c r="F17" s="7"/>
     </row>
     <row r="18" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="19"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="9"/>
-      <c r="E18" s="64"/>
+      <c r="E18" s="55"/>
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="19"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
       <c r="D19" s="9"/>
-      <c r="E19" s="64"/>
+      <c r="E19" s="55"/>
       <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="19"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
       <c r="D20" s="9"/>
-      <c r="E20" s="64"/>
+      <c r="E20" s="55"/>
       <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="19"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
+      <c r="A21" s="18"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
       <c r="D21" s="9"/>
-      <c r="E21" s="64"/>
+      <c r="E21" s="55"/>
       <c r="F21" s="9"/>
     </row>
     <row r="22" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="19"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
+      <c r="A22" s="18"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
       <c r="D22" s="9"/>
-      <c r="E22" s="64"/>
+      <c r="E22" s="55"/>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="19"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
+      <c r="A23" s="18"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
       <c r="D23" s="9"/>
-      <c r="E23" s="64"/>
+      <c r="E23" s="55"/>
       <c r="F23" s="9"/>
     </row>
     <row r="24" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="19"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
+      <c r="A24" s="18"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
       <c r="D24" s="9"/>
-      <c r="E24" s="64"/>
+      <c r="E24" s="55"/>
       <c r="F24" s="9"/>
     </row>
     <row r="25" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="19"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
       <c r="D25" s="9"/>
-      <c r="E25" s="64"/>
+      <c r="E25" s="55"/>
       <c r="F25" s="9"/>
     </row>
     <row r="26" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="19"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
       <c r="D26" s="9"/>
-      <c r="E26" s="64"/>
+      <c r="E26" s="55"/>
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="19"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
       <c r="D27" s="9"/>
-      <c r="E27" s="64"/>
+      <c r="E27" s="55"/>
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="19"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
       <c r="D28" s="9"/>
-      <c r="E28" s="64"/>
+      <c r="E28" s="55"/>
       <c r="F28" s="9"/>
     </row>
     <row r="29" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="19"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
       <c r="D29" s="9"/>
-      <c r="E29" s="64"/>
+      <c r="E29" s="55"/>
       <c r="F29" s="9"/>
     </row>
     <row r="30" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="19"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
       <c r="D30" s="9"/>
-      <c r="E30" s="64"/>
+      <c r="E30" s="55"/>
       <c r="F30" s="9"/>
     </row>
     <row r="31" spans="1:6" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="19"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
       <c r="D31" s="9"/>
-      <c r="E31" s="64"/>
+      <c r="E31" s="55"/>
       <c r="F31" s="9"/>
     </row>
     <row r="32" spans="1:6" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="19"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
       <c r="D32" s="9"/>
-      <c r="E32" s="64"/>
+      <c r="E32" s="55"/>
       <c r="F32" s="9"/>
     </row>
     <row r="33" spans="1:6" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="19"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
       <c r="D33" s="9"/>
-      <c r="E33" s="64"/>
+      <c r="E33" s="55"/>
       <c r="F33" s="9"/>
     </row>
     <row r="34" spans="1:6" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="19"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
       <c r="D34" s="9"/>
-      <c r="E34" s="64"/>
+      <c r="E34" s="55"/>
       <c r="F34" s="9"/>
     </row>
     <row r="35" spans="1:6" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="19"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
       <c r="D35" s="9"/>
-      <c r="E35" s="64"/>
+      <c r="E35" s="55"/>
       <c r="F35" s="9"/>
     </row>
     <row r="36" spans="1:6" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="19"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
       <c r="D36" s="9"/>
-      <c r="E36" s="64"/>
+      <c r="E36" s="55"/>
       <c r="F36" s="9"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.15">
@@ -1595,40 +1584,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="57"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A2" s="66"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A3" s="66"/>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
     </row>
@@ -1641,11 +1630,11 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="67"/>
-      <c r="C6" s="68"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="74"/>
       <c r="D6" s="9" t="s">
         <v>19</v>
       </c>
@@ -1655,10 +1644,10 @@
       <c r="F6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="71" t="s">
+      <c r="G6" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="68"/>
+      <c r="H6" s="74"/>
     </row>
     <row r="7" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="9" t="s">
@@ -1679,240 +1668,240 @@
       <c r="F7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="71" t="s">
+      <c r="G7" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="68"/>
+      <c r="H7" s="74"/>
     </row>
     <row r="8" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="9"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="68"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="74"/>
     </row>
     <row r="9" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="9"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="9"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="71"/>
-      <c r="H9" s="68"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="74"/>
     </row>
     <row r="10" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="9"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="9"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="71"/>
-      <c r="H10" s="68"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="59"/>
+      <c r="H10" s="74"/>
     </row>
     <row r="11" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="9"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="9"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="68"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="59"/>
+      <c r="H11" s="74"/>
     </row>
     <row r="12" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="9"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="9"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="71"/>
-      <c r="H12" s="68"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="74"/>
     </row>
     <row r="13" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="9"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="71"/>
-      <c r="H13" s="68"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="74"/>
     </row>
     <row r="14" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="9"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="9"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="71"/>
-      <c r="H14" s="68"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="59"/>
+      <c r="H14" s="74"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="9"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="9"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="71"/>
-      <c r="H15" s="68"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="59"/>
+      <c r="H15" s="74"/>
     </row>
     <row r="16" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="11"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="9"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="68"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="59"/>
+      <c r="H16" s="74"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="7"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="15"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="69"/>
-      <c r="H17" s="70"/>
+      <c r="E17" s="82"/>
+      <c r="F17" s="82"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="84"/>
     </row>
     <row r="18" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="15"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="70"/>
+      <c r="E18" s="82"/>
+      <c r="F18" s="82"/>
+      <c r="G18" s="83"/>
+      <c r="H18" s="84"/>
     </row>
     <row r="19" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="15"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="69"/>
-      <c r="H19" s="70"/>
+      <c r="E19" s="82"/>
+      <c r="F19" s="82"/>
+      <c r="G19" s="83"/>
+      <c r="H19" s="84"/>
     </row>
     <row r="20" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="9"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="15"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="70"/>
+      <c r="E20" s="82"/>
+      <c r="F20" s="82"/>
+      <c r="G20" s="83"/>
+      <c r="H20" s="84"/>
     </row>
     <row r="21" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="9"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="15"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="70"/>
+      <c r="E21" s="82"/>
+      <c r="F21" s="82"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="84"/>
     </row>
     <row r="22" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="9"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="15"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="69"/>
-      <c r="H22" s="70"/>
+      <c r="E22" s="82"/>
+      <c r="F22" s="82"/>
+      <c r="G22" s="83"/>
+      <c r="H22" s="84"/>
     </row>
     <row r="23" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="9"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="15"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="69"/>
-      <c r="H23" s="70"/>
+      <c r="E23" s="82"/>
+      <c r="F23" s="82"/>
+      <c r="G23" s="83"/>
+      <c r="H23" s="84"/>
     </row>
     <row r="24" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="9"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="15"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="69"/>
-      <c r="H24" s="70"/>
+      <c r="E24" s="82"/>
+      <c r="F24" s="82"/>
+      <c r="G24" s="83"/>
+      <c r="H24" s="84"/>
     </row>
     <row r="25" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="9"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="15"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="69"/>
-      <c r="H25" s="70"/>
+      <c r="E25" s="82"/>
+      <c r="F25" s="82"/>
+      <c r="G25" s="83"/>
+      <c r="H25" s="84"/>
     </row>
     <row r="26" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="9"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="15"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="69"/>
-      <c r="H26" s="70"/>
+      <c r="E26" s="82"/>
+      <c r="F26" s="82"/>
+      <c r="G26" s="83"/>
+      <c r="H26" s="84"/>
     </row>
     <row r="27" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="9"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="15"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="70"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="83"/>
+      <c r="H27" s="84"/>
     </row>
     <row r="28" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="9"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="15"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="69"/>
-      <c r="H28" s="70"/>
+      <c r="E28" s="82"/>
+      <c r="F28" s="82"/>
+      <c r="G28" s="83"/>
+      <c r="H28" s="84"/>
     </row>
     <row r="29" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="9"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="15"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="69"/>
-      <c r="H29" s="70"/>
+      <c r="E29" s="82"/>
+      <c r="F29" s="82"/>
+      <c r="G29" s="83"/>
+      <c r="H29" s="84"/>
     </row>
     <row r="30" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="9"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
       <c r="D30" s="15"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="69"/>
-      <c r="H30" s="70"/>
+      <c r="E30" s="82"/>
+      <c r="F30" s="82"/>
+      <c r="G30" s="83"/>
+      <c r="H30" s="84"/>
     </row>
     <row r="31" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="9"/>
@@ -1921,8 +1910,8 @@
       <c r="D31" s="15"/>
       <c r="E31" s="13"/>
       <c r="F31" s="13"/>
-      <c r="G31" s="69"/>
-      <c r="H31" s="70"/>
+      <c r="G31" s="60"/>
+      <c r="H31" s="61"/>
     </row>
     <row r="32" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="9"/>
@@ -1931,8 +1920,8 @@
       <c r="D32" s="15"/>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
-      <c r="G32" s="69"/>
-      <c r="H32" s="70"/>
+      <c r="G32" s="60"/>
+      <c r="H32" s="61"/>
     </row>
     <row r="33" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="9"/>
@@ -1941,8 +1930,8 @@
       <c r="D33" s="15"/>
       <c r="E33" s="13"/>
       <c r="F33" s="13"/>
-      <c r="G33" s="69"/>
-      <c r="H33" s="70"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="61"/>
     </row>
     <row r="34" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="9"/>
@@ -1951,8 +1940,8 @@
       <c r="D34" s="15"/>
       <c r="E34" s="13"/>
       <c r="F34" s="13"/>
-      <c r="G34" s="69"/>
-      <c r="H34" s="70"/>
+      <c r="G34" s="60"/>
+      <c r="H34" s="61"/>
     </row>
     <row r="35" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="9"/>
@@ -1961,8 +1950,8 @@
       <c r="D35" s="15"/>
       <c r="E35" s="13"/>
       <c r="F35" s="13"/>
-      <c r="G35" s="69"/>
-      <c r="H35" s="70"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="61"/>
     </row>
     <row r="36" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="9"/>
@@ -1971,8 +1960,8 @@
       <c r="D36" s="15"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
-      <c r="G36" s="69"/>
-      <c r="H36" s="70"/>
+      <c r="G36" s="60"/>
+      <c r="H36" s="61"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.15">
       <c r="E37" t="s">
@@ -1980,16 +1969,16 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.15">
-      <c r="A40" s="72" t="s">
+      <c r="A40" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="66"/>
-      <c r="C40" s="66"/>
-      <c r="D40" s="65"/>
-      <c r="E40" s="66"/>
-      <c r="F40" s="66"/>
-      <c r="G40" s="66"/>
-      <c r="H40" s="66"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="57"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="58"/>
+      <c r="H40" s="58"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A41" t="s">
@@ -2001,19 +1990,17 @@
       <c r="F41" t="s">
         <v>17</v>
       </c>
-      <c r="G41" s="66"/>
-      <c r="H41" s="66"/>
+      <c r="G41" s="58"/>
+      <c r="H41" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="G29:H29"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="A1:H3"/>
@@ -2025,9 +2012,17 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G21:H21"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="G21:H21"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="G23:H23"/>
@@ -2035,12 +2030,6 @@
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="G29:H29"/>
   </mergeCells>
   <pageMargins left="0.2188976377952756" right="0.18740157480314959" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="97" fitToHeight="0" orientation="portrait"/>
@@ -2064,40 +2053,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A2" s="66"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
+      <c r="A2" s="58"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
-      <c r="A3" s="66"/>
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
+      <c r="A3" s="58"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
     </row>
@@ -2110,13 +2099,13 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="67" t="s">
+      <c r="B6" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="68"/>
+      <c r="C6" s="81"/>
       <c r="D6" s="8" t="s">
         <v>31</v>
       </c>
@@ -2126,13 +2115,13 @@
       <c r="F6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="78" t="s">
+      <c r="G6" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="68"/>
+      <c r="H6" s="81"/>
     </row>
     <row r="7" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="9" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="10" t="s">
@@ -2141,309 +2130,309 @@
       <c r="C7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="G7" s="71" t="s">
+      <c r="G7" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="68"/>
+      <c r="H7" s="81"/>
     </row>
     <row r="8" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="4"/>
+      <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="68"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="56"/>
+      <c r="H8" s="81"/>
     </row>
     <row r="9" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="4"/>
+      <c r="A9" s="9"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="71"/>
-      <c r="H9" s="68"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="81"/>
     </row>
     <row r="10" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="4"/>
+      <c r="A10" s="9"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="71"/>
-      <c r="H10" s="68"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="81"/>
     </row>
     <row r="11" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="4"/>
+      <c r="A11" s="9"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="68"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="56"/>
+      <c r="H11" s="81"/>
     </row>
     <row r="12" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="4"/>
+      <c r="A12" s="71"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="75"/>
-      <c r="H12" s="76"/>
+      <c r="D12" s="72"/>
+      <c r="E12" s="72"/>
+      <c r="F12" s="72"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="78"/>
     </row>
     <row r="13" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="4"/>
+      <c r="A13" s="71"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="73"/>
-      <c r="H13" s="74"/>
+      <c r="D13" s="73"/>
+      <c r="E13" s="73"/>
+      <c r="F13" s="73"/>
+      <c r="G13" s="79"/>
+      <c r="H13" s="80"/>
     </row>
     <row r="14" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="4"/>
+      <c r="A14" s="71"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="73"/>
-      <c r="H14" s="74"/>
+      <c r="D14" s="73"/>
+      <c r="E14" s="73"/>
+      <c r="F14" s="73"/>
+      <c r="G14" s="79"/>
+      <c r="H14" s="80"/>
     </row>
     <row r="15" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="4"/>
+      <c r="A15" s="71"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="74"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="79"/>
+      <c r="H15" s="80"/>
     </row>
     <row r="16" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="4"/>
+      <c r="A16" s="71"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="73"/>
-      <c r="H16" s="74"/>
+      <c r="D16" s="73"/>
+      <c r="E16" s="73"/>
+      <c r="F16" s="73"/>
+      <c r="G16" s="79"/>
+      <c r="H16" s="80"/>
     </row>
     <row r="17" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="4"/>
+      <c r="A17" s="71"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="73"/>
-      <c r="H17" s="74"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
+      <c r="F17" s="73"/>
+      <c r="G17" s="79"/>
+      <c r="H17" s="80"/>
     </row>
     <row r="18" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="12"/>
+      <c r="A18" s="72"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
-      <c r="G18" s="79"/>
-      <c r="H18" s="74"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="80"/>
     </row>
     <row r="19" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="4"/>
+      <c r="A19" s="71"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="73"/>
-      <c r="H19" s="74"/>
+      <c r="D19" s="73"/>
+      <c r="E19" s="73"/>
+      <c r="F19" s="73"/>
+      <c r="G19" s="79"/>
+      <c r="H19" s="80"/>
     </row>
     <row r="20" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="4"/>
+      <c r="A20" s="71"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="73"/>
-      <c r="H20" s="74"/>
+      <c r="D20" s="73"/>
+      <c r="E20" s="73"/>
+      <c r="F20" s="73"/>
+      <c r="G20" s="79"/>
+      <c r="H20" s="80"/>
     </row>
     <row r="21" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="4"/>
+      <c r="A21" s="71"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="73"/>
-      <c r="H21" s="74"/>
+      <c r="D21" s="73"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="73"/>
+      <c r="G21" s="79"/>
+      <c r="H21" s="80"/>
     </row>
     <row r="22" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="4"/>
+      <c r="A22" s="71"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="73"/>
-      <c r="H22" s="74"/>
+      <c r="D22" s="73"/>
+      <c r="E22" s="73"/>
+      <c r="F22" s="73"/>
+      <c r="G22" s="79"/>
+      <c r="H22" s="80"/>
     </row>
     <row r="23" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="4"/>
+      <c r="A23" s="71"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="73"/>
-      <c r="H23" s="74"/>
+      <c r="D23" s="73"/>
+      <c r="E23" s="73"/>
+      <c r="F23" s="73"/>
+      <c r="G23" s="79"/>
+      <c r="H23" s="80"/>
     </row>
     <row r="24" spans="1:8" s="14" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="4"/>
+      <c r="A24" s="71"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="73"/>
-      <c r="H24" s="74"/>
+      <c r="D24" s="73"/>
+      <c r="E24" s="73"/>
+      <c r="F24" s="73"/>
+      <c r="G24" s="79"/>
+      <c r="H24" s="80"/>
     </row>
     <row r="25" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="4"/>
+      <c r="A25" s="71"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="77"/>
-      <c r="H25" s="74"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="73"/>
+      <c r="F25" s="73"/>
+      <c r="G25" s="66"/>
+      <c r="H25" s="80"/>
     </row>
     <row r="26" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="4"/>
+      <c r="A26" s="71"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="77"/>
-      <c r="H26" s="74"/>
+      <c r="D26" s="73"/>
+      <c r="E26" s="73"/>
+      <c r="F26" s="73"/>
+      <c r="G26" s="66"/>
+      <c r="H26" s="80"/>
     </row>
     <row r="27" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="4"/>
+      <c r="A27" s="71"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="73"/>
-      <c r="H27" s="74"/>
+      <c r="D27" s="73"/>
+      <c r="E27" s="73"/>
+      <c r="F27" s="73"/>
+      <c r="G27" s="79"/>
+      <c r="H27" s="80"/>
     </row>
     <row r="28" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="77"/>
-      <c r="H28" s="74"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="65"/>
+      <c r="H28" s="64"/>
     </row>
     <row r="29" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4"/>
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="77"/>
-      <c r="H29" s="74"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="64"/>
     </row>
     <row r="30" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="12"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="73"/>
-      <c r="H30" s="74"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="64"/>
     </row>
     <row r="31" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="73"/>
-      <c r="H31" s="74"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="63"/>
+      <c r="H31" s="64"/>
     </row>
     <row r="32" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="12"/>
       <c r="B32" s="10"/>
       <c r="C32" s="10"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="73"/>
-      <c r="H32" s="74"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="64"/>
     </row>
     <row r="33" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="4"/>
       <c r="B33" s="10"/>
       <c r="C33" s="10"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="77"/>
-      <c r="H33" s="74"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="65"/>
+      <c r="H33" s="64"/>
     </row>
     <row r="34" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="12"/>
       <c r="B34" s="10"/>
       <c r="C34" s="10"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="74"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="65"/>
+      <c r="H34" s="64"/>
     </row>
     <row r="35" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="4"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="74"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="64"/>
     </row>
     <row r="36" spans="1:8" ht="20.25" hidden="1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="13"/>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="74"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="64"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.15">
       <c r="F37" t="s">
@@ -2451,16 +2440,16 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.15">
-      <c r="A40" s="72" t="s">
+      <c r="A40" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="B40" s="66"/>
-      <c r="C40" s="66"/>
-      <c r="D40" s="66"/>
-      <c r="E40" s="66"/>
-      <c r="F40" s="66"/>
-      <c r="G40" s="66"/>
-      <c r="H40" s="66"/>
+      <c r="B40" s="58"/>
+      <c r="C40" s="58"/>
+      <c r="D40" s="58"/>
+      <c r="E40" s="58"/>
+      <c r="F40" s="58"/>
+      <c r="G40" s="58"/>
+      <c r="H40" s="58"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A41" t="s">
@@ -2472,19 +2461,17 @@
       <c r="F41" t="s">
         <v>17</v>
       </c>
-      <c r="G41" s="66"/>
-      <c r="H41" s="66"/>
+      <c r="G41" s="58"/>
+      <c r="H41" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G30:H30"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="G29:H29"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="A1:H3"/>
@@ -2496,9 +2483,17 @@
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G21:H21"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="G21:H21"/>
     <mergeCell ref="G27:H27"/>
     <mergeCell ref="G36:H36"/>
     <mergeCell ref="G23:H23"/>
@@ -2506,12 +2501,6 @@
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="G34:H34"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="G29:H29"/>
   </mergeCells>
   <pageMargins left="0.2188976377952756" right="0.18740157480314959" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="85" orientation="landscape"/>
@@ -2523,18 +2512,18 @@
   <sheetPr codeName="Arkusz5">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
     <col min="2" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="8.33203125" customWidth="1"/>
-    <col min="7" max="7" width="13.5" style="21" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="13.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A1" s="5" t="s">
         <v>38</v>
       </c>
@@ -2542,53 +2531,49 @@
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="5"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="5"/>
       <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="5"/>
       <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-    </row>
-    <row r="6" spans="1:9" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="6" spans="1:8" ht="27.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="78" t="s">
+      <c r="B6" s="56" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="68"/>
+      <c r="C6" s="74"/>
       <c r="D6" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="75" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="24"/>
-      <c r="G6" s="27" t="s">
+      <c r="F6" s="21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A7" s="9" t="s">
         <v>23</v>
       </c>
@@ -2601,274 +2586,244 @@
       <c r="D7" s="16">
         <v>1</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="76" t="s">
         <v>43</v>
       </c>
-      <c r="F7" s="25"/>
-      <c r="G7" s="28" t="s">
+      <c r="F7" s="22" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="16"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="28"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E8" s="76"/>
+      <c r="F8" s="22"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A9" s="9"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="16"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="28"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E9" s="76"/>
+      <c r="F9" s="22"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A10" s="9"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
       <c r="D10" s="16"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="28"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E10" s="76"/>
+      <c r="F10" s="22"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A11" s="9"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
       <c r="D11" s="16"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="28"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E11" s="76"/>
+      <c r="F11" s="22"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A12" s="9"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="28"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E12" s="76"/>
+      <c r="F12" s="22"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A13" s="9"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="16"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="28"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E13" s="76"/>
+      <c r="F13" s="22"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A14" s="9"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="16"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="28"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E14" s="76"/>
+      <c r="F14" s="22"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A15" s="9"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="16"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="28"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="E15" s="76"/>
+      <c r="F15" s="22"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
       <c r="A16" s="9"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="16"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="28"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E16" s="76"/>
+      <c r="F16" s="22"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A17" s="9"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="16"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="28"/>
-    </row>
-    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="E17" s="76"/>
+      <c r="F17" s="22"/>
+    </row>
+    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="16"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="28"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E18" s="76"/>
+      <c r="F18" s="22"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A19" s="9"/>
       <c r="B19" s="10"/>
       <c r="C19" s="10"/>
       <c r="D19" s="16"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="28"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E19" s="76"/>
+      <c r="F19" s="22"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A20" s="9"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="16"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="28"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E20" s="76"/>
+      <c r="F20" s="22"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A21" s="9"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
       <c r="D21" s="16"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="28"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E21" s="76"/>
+      <c r="F21" s="22"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A22" s="9"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="16"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="28"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E22" s="76"/>
+      <c r="F22" s="22"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A23" s="9"/>
       <c r="B23" s="10"/>
       <c r="C23" s="10"/>
       <c r="D23" s="16"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="28"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E23" s="76"/>
+      <c r="F23" s="22"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A24" s="9"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="16"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="28"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E24" s="76"/>
+      <c r="F24" s="22"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A25" s="9"/>
       <c r="B25" s="10"/>
       <c r="C25" s="10"/>
       <c r="D25" s="16"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="28"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E25" s="76"/>
+      <c r="F25" s="22"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A26" s="9"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="16"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="28"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E26" s="76"/>
+      <c r="F26" s="22"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A27" s="9"/>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
       <c r="D27" s="16"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="28"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="E27" s="76"/>
+      <c r="F27" s="22"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A28" s="11"/>
-      <c r="B28" s="50"/>
-      <c r="C28" s="50"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="53"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="46"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A29" s="7"/>
-      <c r="B29" s="58"/>
-      <c r="C29" s="58"/>
-      <c r="D29" s="59"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="61"/>
-      <c r="G29" s="28"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B29" s="51"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="22"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A30" s="7"/>
-      <c r="B30" s="58"/>
-      <c r="C30" s="58"/>
-      <c r="D30" s="59"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="61"/>
-      <c r="G30" s="28"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="22"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A31" s="6"/>
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="56"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="57"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B31" s="47"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="50"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A32" s="6"/>
-      <c r="B32" s="54"/>
-      <c r="C32" s="54"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="56"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="57"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B32" s="47"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="50"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A33" s="6"/>
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="56"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="57"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B33" s="47"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="50"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A34" s="6"/>
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="56"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="57"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="50"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A35" s="6"/>
-      <c r="B35" s="54"/>
-      <c r="C35" s="54"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="56"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="57"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.15">
+      <c r="B35" s="47"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="50"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A36" s="6"/>
-      <c r="B36" s="54"/>
-      <c r="C36" s="54"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="57"/>
+      <c r="B36" s="47"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2892,19 +2847,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A1" s="29"/>
-      <c r="B1" s="72" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.15">
       <c r="B3" t="s">
@@ -2912,637 +2867,637 @@
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="C4" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="33" t="s">
+      <c r="D4" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="33" t="s">
+      <c r="E4" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="33" t="s">
+      <c r="F4" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="H4" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="I4" s="33" t="s">
+      <c r="I4" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="J4" s="33" t="s">
+      <c r="J4" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="K4" s="33" t="s">
+      <c r="K4" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="L4" s="33" t="s">
+      <c r="L4" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="M4" s="34" t="s">
+      <c r="M4" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="N4" s="35" t="s">
+      <c r="N4" s="29" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="37">
+      <c r="B5" s="31">
         <v>45912</v>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="32">
         <v>1</v>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="32">
         <v>2</v>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="32">
         <v>3</v>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="32">
         <v>4</v>
       </c>
-      <c r="G5" s="38">
+      <c r="G5" s="32">
         <v>5</v>
       </c>
-      <c r="H5" s="38">
+      <c r="H5" s="32">
         <v>6</v>
       </c>
-      <c r="I5" s="38">
+      <c r="I5" s="32">
         <v>7</v>
       </c>
-      <c r="J5" s="38">
+      <c r="J5" s="32">
         <v>8</v>
       </c>
-      <c r="K5" s="38">
+      <c r="K5" s="32">
         <v>9</v>
       </c>
-      <c r="L5" s="38">
+      <c r="L5" s="32">
         <v>10</v>
       </c>
-      <c r="M5" s="38">
+      <c r="M5" s="32">
         <v>11</v>
       </c>
-      <c r="N5" s="39"/>
+      <c r="N5" s="33"/>
     </row>
     <row r="6" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="37">
+      <c r="B6" s="31">
         <v>45913</v>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="32">
         <v>12</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="32">
         <v>13</v>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="32">
         <v>14</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="32">
         <v>15</v>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="32">
         <v>16</v>
       </c>
-      <c r="H6" s="38">
+      <c r="H6" s="32">
         <v>17</v>
       </c>
-      <c r="I6" s="38">
+      <c r="I6" s="32">
         <v>18</v>
       </c>
-      <c r="J6" s="38">
+      <c r="J6" s="32">
         <v>19</v>
       </c>
-      <c r="K6" s="38">
+      <c r="K6" s="32">
         <v>20</v>
       </c>
-      <c r="L6" s="38">
+      <c r="L6" s="32">
         <v>21</v>
       </c>
-      <c r="M6" s="38">
+      <c r="M6" s="32">
         <v>22</v>
       </c>
-      <c r="N6" s="39"/>
+      <c r="N6" s="33"/>
     </row>
     <row r="7" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="37">
+      <c r="B7" s="31">
         <v>45914</v>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="32">
         <v>23</v>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="32">
         <v>24</v>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="32">
         <v>25</v>
       </c>
-      <c r="F7" s="38">
+      <c r="F7" s="32">
         <v>26</v>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="32">
         <v>27</v>
       </c>
-      <c r="H7" s="38">
+      <c r="H7" s="32">
         <v>28</v>
       </c>
-      <c r="I7" s="38">
+      <c r="I7" s="32">
         <v>29</v>
       </c>
-      <c r="J7" s="38">
+      <c r="J7" s="32">
         <v>30</v>
       </c>
-      <c r="K7" s="38">
+      <c r="K7" s="32">
         <v>31</v>
       </c>
-      <c r="L7" s="38">
+      <c r="L7" s="32">
         <v>32</v>
       </c>
-      <c r="M7" s="38">
+      <c r="M7" s="32">
         <v>33</v>
       </c>
-      <c r="N7" s="39"/>
+      <c r="N7" s="33"/>
     </row>
     <row r="8" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="37">
+      <c r="B8" s="31">
         <v>45926</v>
       </c>
-      <c r="C8" s="38">
+      <c r="C8" s="32">
         <v>34</v>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="32">
         <v>35</v>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="32">
         <v>36</v>
       </c>
-      <c r="F8" s="38">
+      <c r="F8" s="32">
         <v>37</v>
       </c>
-      <c r="G8" s="38">
+      <c r="G8" s="32">
         <v>38</v>
       </c>
-      <c r="H8" s="38">
+      <c r="H8" s="32">
         <v>39</v>
       </c>
-      <c r="I8" s="38">
+      <c r="I8" s="32">
         <v>40</v>
       </c>
-      <c r="J8" s="38">
+      <c r="J8" s="32">
         <v>41</v>
       </c>
-      <c r="K8" s="38">
+      <c r="K8" s="32">
         <v>42</v>
       </c>
-      <c r="L8" s="38">
+      <c r="L8" s="32">
         <v>43</v>
       </c>
-      <c r="M8" s="38">
+      <c r="M8" s="32">
         <v>44</v>
       </c>
-      <c r="N8" s="39"/>
+      <c r="N8" s="33"/>
     </row>
     <row r="9" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="B9" s="37">
+      <c r="B9" s="31">
         <v>45927</v>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="32">
         <v>45</v>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="32">
         <v>46</v>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="32">
         <v>47</v>
       </c>
-      <c r="F9" s="38">
+      <c r="F9" s="32">
         <v>48</v>
       </c>
-      <c r="G9" s="38">
+      <c r="G9" s="32">
         <v>49</v>
       </c>
-      <c r="H9" s="38">
+      <c r="H9" s="32">
         <v>50</v>
       </c>
-      <c r="I9" s="38">
+      <c r="I9" s="32">
         <v>51</v>
       </c>
-      <c r="J9" s="38">
+      <c r="J9" s="32">
         <v>52</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="32">
         <v>53</v>
       </c>
-      <c r="L9" s="38">
+      <c r="L9" s="32">
         <v>54</v>
       </c>
-      <c r="M9" s="38">
+      <c r="M9" s="32">
         <v>55</v>
       </c>
-      <c r="N9" s="39"/>
+      <c r="N9" s="33"/>
     </row>
     <row r="10" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="31">
         <v>45928</v>
       </c>
-      <c r="C10" s="38">
+      <c r="C10" s="32">
         <v>56</v>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="32">
         <v>57</v>
       </c>
-      <c r="E10" s="38">
+      <c r="E10" s="32">
         <v>58</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="32">
         <v>59</v>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="32">
         <v>60</v>
       </c>
-      <c r="H10" s="38">
+      <c r="H10" s="32">
         <v>61</v>
       </c>
-      <c r="I10" s="38">
+      <c r="I10" s="32">
         <v>62</v>
       </c>
-      <c r="J10" s="38">
+      <c r="J10" s="32">
         <v>63</v>
       </c>
-      <c r="K10" s="38">
+      <c r="K10" s="32">
         <v>64</v>
       </c>
-      <c r="L10" s="38">
+      <c r="L10" s="32">
         <v>65</v>
       </c>
-      <c r="M10" s="38">
+      <c r="M10" s="32">
         <v>66</v>
       </c>
-      <c r="N10" s="39"/>
+      <c r="N10" s="33"/>
     </row>
     <row r="11" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="41">
+      <c r="B11" s="35">
         <f>B10</f>
         <v>45928</v>
       </c>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-      <c r="K11" s="42"/>
-      <c r="L11" s="42"/>
-      <c r="M11" s="43"/>
-      <c r="N11" s="44"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="36"/>
+      <c r="K11" s="36"/>
+      <c r="L11" s="36"/>
+      <c r="M11" s="37"/>
+      <c r="N11" s="38"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A13" s="80" t="s">
+      <c r="A13" s="67" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="66"/>
-      <c r="C13" s="66"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="66"/>
-      <c r="F13" s="66"/>
-      <c r="G13" s="66"/>
-      <c r="H13" s="66"/>
-      <c r="I13" s="66"/>
-      <c r="J13" s="66"/>
-      <c r="K13" s="66"/>
-      <c r="L13" s="66"/>
-      <c r="M13" s="66"/>
-      <c r="N13" s="66"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+      <c r="H13" s="58"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="58"/>
+      <c r="K13" s="58"/>
+      <c r="L13" s="58"/>
+      <c r="M13" s="58"/>
+      <c r="N13" s="58"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A14" s="66"/>
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="66"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="66"/>
-      <c r="K14" s="66"/>
-      <c r="L14" s="66"/>
-      <c r="M14" s="66"/>
-      <c r="N14" s="66"/>
+      <c r="A14" s="58"/>
+      <c r="B14" s="58"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="58"/>
+      <c r="E14" s="58"/>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58"/>
+      <c r="H14" s="58"/>
+      <c r="I14" s="58"/>
+      <c r="J14" s="58"/>
+      <c r="K14" s="58"/>
+      <c r="L14" s="58"/>
+      <c r="M14" s="58"/>
+      <c r="N14" s="58"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A15" s="66"/>
-      <c r="B15" s="66"/>
-      <c r="C15" s="66"/>
-      <c r="D15" s="66"/>
-      <c r="E15" s="66"/>
-      <c r="F15" s="66"/>
-      <c r="G15" s="66"/>
-      <c r="H15" s="66"/>
-      <c r="I15" s="66"/>
-      <c r="J15" s="66"/>
-      <c r="K15" s="66"/>
-      <c r="L15" s="66"/>
-      <c r="M15" s="66"/>
-      <c r="N15" s="66"/>
+      <c r="A15" s="58"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58"/>
+      <c r="H15" s="58"/>
+      <c r="I15" s="58"/>
+      <c r="J15" s="58"/>
+      <c r="K15" s="58"/>
+      <c r="L15" s="58"/>
+      <c r="M15" s="58"/>
+      <c r="N15" s="58"/>
     </row>
     <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="45"/>
-      <c r="B16" s="45"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="46"/>
-      <c r="F16" s="46"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="46"/>
-      <c r="I16" s="46"/>
-      <c r="J16" s="46"/>
-      <c r="K16" s="46"/>
-      <c r="L16" s="46"/>
-      <c r="M16" s="46"/>
-      <c r="N16" s="46"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="39"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="40"/>
+      <c r="K16" s="40"/>
+      <c r="L16" s="40"/>
+      <c r="M16" s="40"/>
+      <c r="N16" s="40"/>
     </row>
     <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="45"/>
-      <c r="B17" s="45"/>
-      <c r="C17" s="45"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="46"/>
-      <c r="F17" s="46"/>
-      <c r="G17" s="48">
+      <c r="A17" s="39"/>
+      <c r="B17" s="39"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="42">
         <f>B5</f>
         <v>45912</v>
       </c>
-      <c r="H17" s="81" t="s">
+      <c r="H17" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="I17" s="66"/>
-      <c r="J17" s="66"/>
-      <c r="K17" s="66"/>
-      <c r="L17" s="66"/>
-      <c r="M17" s="66"/>
-      <c r="N17" s="66"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="58"/>
+      <c r="K17" s="58"/>
+      <c r="L17" s="58"/>
+      <c r="M17" s="58"/>
+      <c r="N17" s="58"/>
     </row>
     <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="46"/>
-      <c r="B18" s="46"/>
-      <c r="C18" s="46"/>
-      <c r="D18" s="46"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
-      <c r="I18" s="46"/>
-      <c r="J18" s="46"/>
-      <c r="K18" s="46"/>
-      <c r="L18" s="46"/>
-      <c r="M18" s="46"/>
-      <c r="N18" s="46"/>
+      <c r="A18" s="40"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A19" s="83" t="s">
+      <c r="A19" s="70" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="66"/>
-      <c r="C19" s="66"/>
-      <c r="D19" s="66"/>
-      <c r="E19" s="66"/>
-      <c r="F19" s="66"/>
-      <c r="G19" s="66"/>
-      <c r="H19" s="66"/>
-      <c r="I19" s="66"/>
-      <c r="J19" s="66"/>
-      <c r="K19" s="66"/>
-      <c r="L19" s="66"/>
-      <c r="M19" s="66"/>
-      <c r="N19" s="66"/>
+      <c r="B19" s="58"/>
+      <c r="C19" s="58"/>
+      <c r="D19" s="58"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58"/>
+      <c r="H19" s="58"/>
+      <c r="I19" s="58"/>
+      <c r="J19" s="58"/>
+      <c r="K19" s="58"/>
+      <c r="L19" s="58"/>
+      <c r="M19" s="58"/>
+      <c r="N19" s="58"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A20" s="66"/>
-      <c r="B20" s="66"/>
-      <c r="C20" s="66"/>
-      <c r="D20" s="66"/>
-      <c r="E20" s="66"/>
-      <c r="F20" s="66"/>
-      <c r="G20" s="66"/>
-      <c r="H20" s="66"/>
-      <c r="I20" s="66"/>
-      <c r="J20" s="66"/>
-      <c r="K20" s="66"/>
-      <c r="L20" s="66"/>
-      <c r="M20" s="66"/>
-      <c r="N20" s="66"/>
+      <c r="A20" s="58"/>
+      <c r="B20" s="58"/>
+      <c r="C20" s="58"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58"/>
+      <c r="H20" s="58"/>
+      <c r="I20" s="58"/>
+      <c r="J20" s="58"/>
+      <c r="K20" s="58"/>
+      <c r="L20" s="58"/>
+      <c r="M20" s="58"/>
+      <c r="N20" s="58"/>
     </row>
     <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="47"/>
-      <c r="B21" s="47"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="49">
+      <c r="A21" s="41"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="43">
         <f>B5</f>
         <v>45912</v>
       </c>
-      <c r="H21" s="81" t="s">
+      <c r="H21" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="I21" s="66"/>
-      <c r="J21" s="66"/>
-      <c r="K21" s="66"/>
-      <c r="L21" s="66"/>
-      <c r="M21" s="66"/>
-      <c r="N21" s="66"/>
+      <c r="I21" s="58"/>
+      <c r="J21" s="58"/>
+      <c r="K21" s="58"/>
+      <c r="L21" s="58"/>
+      <c r="M21" s="58"/>
+      <c r="N21" s="58"/>
     </row>
     <row r="22" spans="1:14" ht="42.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="80" t="s">
+      <c r="A22" s="67" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="66"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="66"/>
-      <c r="I22" s="66"/>
-      <c r="J22" s="66"/>
-      <c r="K22" s="66"/>
-      <c r="L22" s="66"/>
-      <c r="M22" s="66"/>
-      <c r="N22" s="66"/>
+      <c r="B22" s="58"/>
+      <c r="C22" s="58"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="58"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58"/>
+      <c r="H22" s="58"/>
+      <c r="I22" s="58"/>
+      <c r="J22" s="58"/>
+      <c r="K22" s="58"/>
+      <c r="L22" s="58"/>
+      <c r="M22" s="58"/>
+      <c r="N22" s="58"/>
     </row>
     <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="47"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="48">
+      <c r="A23" s="41"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="42">
         <f>B5</f>
         <v>45912</v>
       </c>
-      <c r="H23" s="81" t="s">
+      <c r="H23" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
-      <c r="K23" s="66"/>
-      <c r="L23" s="66"/>
-      <c r="M23" s="66"/>
-      <c r="N23" s="66"/>
+      <c r="I23" s="58"/>
+      <c r="J23" s="58"/>
+      <c r="K23" s="58"/>
+      <c r="L23" s="58"/>
+      <c r="M23" s="58"/>
+      <c r="N23" s="58"/>
     </row>
     <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="46"/>
-      <c r="K24" s="46"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="46"/>
-      <c r="N24" s="46"/>
+      <c r="A24" s="40"/>
+      <c r="B24" s="40"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="40"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="40"/>
+      <c r="J24" s="40"/>
+      <c r="K24" s="40"/>
+      <c r="L24" s="40"/>
+      <c r="M24" s="40"/>
+      <c r="N24" s="40"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A25" s="82" t="s">
+      <c r="A25" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="B25" s="66"/>
-      <c r="C25" s="66"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="66"/>
-      <c r="F25" s="66"/>
-      <c r="G25" s="66"/>
-      <c r="H25" s="66"/>
-      <c r="I25" s="66"/>
-      <c r="J25" s="66"/>
-      <c r="K25" s="66"/>
-      <c r="L25" s="66"/>
-      <c r="M25" s="66"/>
-      <c r="N25" s="66"/>
+      <c r="B25" s="58"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="58"/>
+      <c r="E25" s="58"/>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58"/>
+      <c r="H25" s="58"/>
+      <c r="I25" s="58"/>
+      <c r="J25" s="58"/>
+      <c r="K25" s="58"/>
+      <c r="L25" s="58"/>
+      <c r="M25" s="58"/>
+      <c r="N25" s="58"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A26" s="66"/>
-      <c r="B26" s="66"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="66"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="66"/>
-      <c r="J26" s="66"/>
-      <c r="K26" s="66"/>
-      <c r="L26" s="66"/>
-      <c r="M26" s="66"/>
-      <c r="N26" s="66"/>
+      <c r="A26" s="58"/>
+      <c r="B26" s="58"/>
+      <c r="C26" s="58"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="58"/>
+      <c r="L26" s="58"/>
+      <c r="M26" s="58"/>
+      <c r="N26" s="58"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A27" s="66"/>
-      <c r="B27" s="66"/>
-      <c r="C27" s="66"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="66"/>
-      <c r="F27" s="66"/>
-      <c r="G27" s="66"/>
-      <c r="H27" s="66"/>
-      <c r="I27" s="66"/>
-      <c r="J27" s="66"/>
-      <c r="K27" s="66"/>
-      <c r="L27" s="66"/>
-      <c r="M27" s="66"/>
-      <c r="N27" s="66"/>
+      <c r="A27" s="58"/>
+      <c r="B27" s="58"/>
+      <c r="C27" s="58"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="58"/>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58"/>
+      <c r="H27" s="58"/>
+      <c r="I27" s="58"/>
+      <c r="J27" s="58"/>
+      <c r="K27" s="58"/>
+      <c r="L27" s="58"/>
+      <c r="M27" s="58"/>
+      <c r="N27" s="58"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.15">
-      <c r="A28" s="66"/>
-      <c r="B28" s="66"/>
-      <c r="C28" s="66"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
-      <c r="F28" s="66"/>
-      <c r="G28" s="66"/>
-      <c r="H28" s="66"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="66"/>
-      <c r="K28" s="66"/>
-      <c r="L28" s="66"/>
-      <c r="M28" s="66"/>
-      <c r="N28" s="66"/>
+      <c r="A28" s="58"/>
+      <c r="B28" s="58"/>
+      <c r="C28" s="58"/>
+      <c r="D28" s="58"/>
+      <c r="E28" s="58"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58"/>
+      <c r="H28" s="58"/>
+      <c r="I28" s="58"/>
+      <c r="J28" s="58"/>
+      <c r="K28" s="58"/>
+      <c r="L28" s="58"/>
+      <c r="M28" s="58"/>
+      <c r="N28" s="58"/>
     </row>
     <row r="29" spans="1:14" ht="27.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="66"/>
-      <c r="B29" s="66"/>
-      <c r="C29" s="66"/>
-      <c r="D29" s="66"/>
-      <c r="E29" s="66"/>
-      <c r="F29" s="66"/>
-      <c r="G29" s="66"/>
-      <c r="H29" s="66"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="66"/>
-      <c r="K29" s="66"/>
-      <c r="L29" s="66"/>
-      <c r="M29" s="66"/>
-      <c r="N29" s="66"/>
+      <c r="A29" s="58"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="58"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="58"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="58"/>
+      <c r="K29" s="58"/>
+      <c r="L29" s="58"/>
+      <c r="M29" s="58"/>
+      <c r="N29" s="58"/>
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="46"/>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="48">
+      <c r="A30" s="40"/>
+      <c r="B30" s="40"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="42">
         <f>B5</f>
         <v>45912</v>
       </c>
-      <c r="H30" s="81" t="s">
+      <c r="H30" s="68" t="s">
         <v>69</v>
       </c>
-      <c r="I30" s="66"/>
-      <c r="J30" s="66"/>
-      <c r="K30" s="66"/>
-      <c r="L30" s="66"/>
-      <c r="M30" s="66"/>
-      <c r="N30" s="66"/>
+      <c r="I30" s="58"/>
+      <c r="J30" s="58"/>
+      <c r="K30" s="58"/>
+      <c r="L30" s="58"/>
+      <c r="M30" s="58"/>
+      <c r="N30" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>